<commit_message>
feat: add semester 1 courses and update schedule documentation
</commit_message>
<xml_diff>
--- a/data/jadwal_zoom.xlsx
+++ b/data/jadwal_zoom.xlsx
@@ -486,7 +486,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E35"/>
+  <dimension ref="A1:E38"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -507,16 +507,16 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B2" t="str">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C2" t="str">
-        <v>2024 - TS 3325 / 03</v>
+        <v>PU 1206</v>
       </c>
       <c r="D2" t="str">
-        <v>Matematika III</v>
+        <v>Matematika I</v>
       </c>
       <c r="E2" t="str">
         <v>Dra. MARAMA NAMORA, M.T.</v>
@@ -524,36 +524,36 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B3" t="str">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C3" t="str">
-        <v>2024 - TS 3326 / 03</v>
+        <v>PU 1209</v>
       </c>
       <c r="D3" t="str">
-        <v>Fisika II</v>
+        <v>Logika Teknologi dan Transformasi Digital (Internet of Things)</v>
       </c>
       <c r="E3" t="str">
-        <v>Dra. RADEN RORO HERLIANI, Msi</v>
+        <v>MUHAMMAD FAIZ SYAIFUL ISLAM, M.Si.</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B4" t="str">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C4" t="str">
-        <v>2024 - TS 3327 / 03</v>
+        <v>PU 1210</v>
       </c>
       <c r="D4" t="str">
-        <v>Kimia Dasar</v>
+        <v>Etika Profesi dan Pendidikan Anti Korupsi</v>
       </c>
       <c r="E4" t="str">
-        <v>Dr. TULUS SUKRENI, S.T.,M.T.</v>
+        <v>Drs. GUNAWAN WIBISONO, M.T.</v>
       </c>
     </row>
     <row r="5">
@@ -564,13 +564,13 @@
         <v>3</v>
       </c>
       <c r="C5" t="str">
-        <v>2024 - TS 3328 / 03</v>
+        <v>TS 3325</v>
       </c>
       <c r="D5" t="str">
-        <v>Mekanika Bahan</v>
+        <v>Matematika III</v>
       </c>
       <c r="E5" t="str">
-        <v>BAMBANG TRIGUNO, S.T., M.T.</v>
+        <v>Dra. MARAMA NAMORA, M.T.</v>
       </c>
     </row>
     <row r="6">
@@ -581,13 +581,13 @@
         <v>3</v>
       </c>
       <c r="C6" t="str">
-        <v>2024 - TS 3329 / 03</v>
+        <v>TS 3326</v>
       </c>
       <c r="D6" t="str">
-        <v>Mekanika Tanah I</v>
+        <v>Fisika II</v>
       </c>
       <c r="E6" t="str">
-        <v>Dr Ir MUKTAR NAPITUPULU, M.Sc</v>
+        <v>Dra. RADEN RORO HERLIANI, Msi</v>
       </c>
     </row>
     <row r="7">
@@ -598,13 +598,13 @@
         <v>3</v>
       </c>
       <c r="C7" t="str">
-        <v>2024 - TS 3330 / 03</v>
+        <v>TS 3327</v>
       </c>
       <c r="D7" t="str">
-        <v>Pengelolaan Sumber Daya Air</v>
+        <v>Kimia Dasar</v>
       </c>
       <c r="E7" t="str">
-        <v>Dr. DUKI MALINDO, S.T., M.Const.Mgt.</v>
+        <v>Dr. TULUS SUKRENI, S.T.,M.T.</v>
       </c>
     </row>
     <row r="8">
@@ -615,13 +615,13 @@
         <v>3</v>
       </c>
       <c r="C8" t="str">
-        <v>2024 - TS 3331 / 03</v>
+        <v>TS 3328</v>
       </c>
       <c r="D8" t="str">
-        <v>Hidrologi Terapan</v>
+        <v>Mekanika Bahan</v>
       </c>
       <c r="E8" t="str">
-        <v>ELLY NORIZA, S.T., M.A.</v>
+        <v>BAMBANG TRIGUNO, S.T., M.T.</v>
       </c>
     </row>
     <row r="9">
@@ -632,13 +632,13 @@
         <v>3</v>
       </c>
       <c r="C9" t="str">
-        <v>2024 - TS 3332 / 03</v>
+        <v>TS 3329</v>
       </c>
       <c r="D9" t="str">
-        <v>Transportasi &amp; Rekayasa Lalu Lintas</v>
+        <v>Mekanika Tanah I</v>
       </c>
       <c r="E9" t="str">
-        <v>Dr. Ir. BUDIAMIN, S.T., M.T., IPM</v>
+        <v>Dr Ir MUKTAR NAPITUPULU, M.Sc</v>
       </c>
     </row>
     <row r="10">
@@ -649,13 +649,13 @@
         <v>3</v>
       </c>
       <c r="C10" t="str">
-        <v>2024 - TS 3333 / 03</v>
+        <v>TS 3330</v>
       </c>
       <c r="D10" t="str">
-        <v>Struktur Bangunan</v>
+        <v>Pengelolaan Sumber Daya Air</v>
       </c>
       <c r="E10" t="str">
-        <v>Dr. Ir. SYAHPUTRA A GANI, S.T., M.T., IPU.</v>
+        <v>Dr. DUKI MALINDO, S.T., M.Const.Mgt.</v>
       </c>
     </row>
     <row r="11">
@@ -666,64 +666,64 @@
         <v>3</v>
       </c>
       <c r="C11" t="str">
-        <v>2024 - TS 3334 / 03</v>
+        <v>TS 3331</v>
       </c>
       <c r="D11" t="str">
-        <v>Surveying dan Sistem Informasi Geografis</v>
+        <v>Hidrologi Terapan</v>
       </c>
       <c r="E11" t="str">
-        <v>ANDIKA SETIAWAN</v>
+        <v>ELLY NORIZA, S.T., M.A.</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="B12" t="str">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C12" t="str">
-        <v>2024 - TS 5345 / 05</v>
+        <v>TS 3332</v>
       </c>
       <c r="D12" t="str">
-        <v>Pemodelan Struktur</v>
+        <v>Transportasi &amp; Rekayasa Lalu Lintas</v>
       </c>
       <c r="E12" t="str">
-        <v>EKO NURLITA WIDAYATI, S.T., M.T.</v>
+        <v>Dr. Ir. BUDIAMIN, S.T., M.T., IPM</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="B13" t="str">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C13" t="str">
-        <v>2024 - TS 5346 / 05</v>
+        <v>TS 3333</v>
       </c>
       <c r="D13" t="str">
-        <v>Praktik Pemodelan Struktur</v>
+        <v>Struktur Bangunan</v>
       </c>
       <c r="E13" t="str">
-        <v>EKO NURLITA WIDAYATI, S.T., M.T.</v>
+        <v>Dr. Ir. SYAHPUTRA A GANI, S.T., M.T., IPU.</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="B14" t="str">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C14" t="str">
-        <v>2024 - TS 5347 / 05</v>
+        <v>TS 3334</v>
       </c>
       <c r="D14" t="str">
-        <v>Rekayasa Struktur Bangunan Beton</v>
+        <v>Surveying dan Sistem Informasi Geografis</v>
       </c>
       <c r="E14" t="str">
-        <v>Drs. GUNAWAN WIBISONO, M.T.</v>
+        <v>ANDIKA SETIAWAN</v>
       </c>
     </row>
     <row r="15">
@@ -734,13 +734,13 @@
         <v>5</v>
       </c>
       <c r="C15" t="str">
-        <v>2024 - TS 5348 / 05</v>
+        <v>TS 5345</v>
       </c>
       <c r="D15" t="str">
-        <v>Rekayasa Struktur Bangunan Baja</v>
+        <v>Pemodelan Struktur</v>
       </c>
       <c r="E15" t="str">
-        <v>SIGIT HIMAWAN, S.T., M.Sc</v>
+        <v>EKO NURLITA WIDAYATI, S.T., M.T.</v>
       </c>
     </row>
     <row r="16">
@@ -751,13 +751,13 @@
         <v>5</v>
       </c>
       <c r="C16" t="str">
-        <v>2024 - TS 5349 / 05</v>
+        <v>TS 5346</v>
       </c>
       <c r="D16" t="str">
-        <v>Desain Fondasi I</v>
+        <v>Praktik Pemodelan Struktur</v>
       </c>
       <c r="E16" t="str">
-        <v>Dr. Drs. HARMADI, ST, Sp1</v>
+        <v>EKO NURLITA WIDAYATI, S.T., M.T.</v>
       </c>
     </row>
     <row r="17">
@@ -768,13 +768,13 @@
         <v>5</v>
       </c>
       <c r="C17" t="str">
-        <v>2024 - TS 5350 / 05</v>
+        <v>TS 5347</v>
       </c>
       <c r="D17" t="str">
-        <v>Rekayasa Perkerasan dan Preservasi Jalan</v>
+        <v>Rekayasa Struktur Bangunan Beton</v>
       </c>
       <c r="E17" t="str">
-        <v>Dr. Ir. BUDIAMIN, S.T., M.T., IPM</v>
+        <v>Drs. GUNAWAN WIBISONO, M.T.</v>
       </c>
     </row>
     <row r="18">
@@ -785,10 +785,10 @@
         <v>5</v>
       </c>
       <c r="C18" t="str">
-        <v>2024 - TS 5351 / 05</v>
+        <v>TS 5348</v>
       </c>
       <c r="D18" t="str">
-        <v>Manajemen Konstruksi</v>
+        <v>Rekayasa Struktur Bangunan Baja</v>
       </c>
       <c r="E18" t="str">
         <v>SIGIT HIMAWAN, S.T., M.Sc</v>
@@ -802,13 +802,13 @@
         <v>5</v>
       </c>
       <c r="C19" t="str">
-        <v>2024 - TS 5352 / 05</v>
+        <v>TS 5349</v>
       </c>
       <c r="D19" t="str">
-        <v>Ekonomi Rekayasa dan Analisis Finansial</v>
+        <v>Desain Fondasi I</v>
       </c>
       <c r="E19" t="str">
-        <v>EKO NURLITA WIDAYATI, S.T., M.T.</v>
+        <v>Dr. Drs. HARMADI, ST, Sp1</v>
       </c>
     </row>
     <row r="20">
@@ -819,13 +819,13 @@
         <v>5</v>
       </c>
       <c r="C20" t="str">
-        <v>2024 - TS 5353 / 05</v>
+        <v>TS 5350</v>
       </c>
       <c r="D20" t="str">
-        <v>Praktikum Beton</v>
+        <v>Rekayasa Perkerasan dan Preservasi Jalan</v>
       </c>
       <c r="E20" t="str">
-        <v>KARTIKA WATI, ST</v>
+        <v>Dr. Ir. BUDIAMIN, S.T., M.T., IPM</v>
       </c>
     </row>
     <row r="21">
@@ -836,13 +836,13 @@
         <v>5</v>
       </c>
       <c r="C21" t="str">
-        <v>2024 - TS 5354 / 05</v>
+        <v>TS 5351</v>
       </c>
       <c r="D21" t="str">
-        <v>Praktikum Surveying dan Sistem Informasi Geografis</v>
+        <v>Manajemen Konstruksi</v>
       </c>
       <c r="E21" t="str">
-        <v>KARTIKA WATI, ST</v>
+        <v>SIGIT HIMAWAN, S.T., M.Sc</v>
       </c>
     </row>
     <row r="22">
@@ -853,13 +853,13 @@
         <v>5</v>
       </c>
       <c r="C22" t="str">
-        <v>2024 - TS 5355 / 05</v>
+        <v>TS 5352</v>
       </c>
       <c r="D22" t="str">
-        <v>Rekayasa Sungai dan Pantai</v>
+        <v>Ekonomi Rekayasa dan Analisis Finansial</v>
       </c>
       <c r="E22" t="str">
-        <v>IIS TRISNAWATI, S.T., M.T.</v>
+        <v>EKO NURLITA WIDAYATI, S.T., M.T.</v>
       </c>
     </row>
     <row r="23">
@@ -870,64 +870,64 @@
         <v>5</v>
       </c>
       <c r="C23" t="str">
-        <v>2024 - TS 5356 / 05</v>
+        <v>TS 5353</v>
       </c>
       <c r="D23" t="str">
-        <v>Rekayasa Irigasi dan Rawa</v>
+        <v>Praktikum Beton</v>
       </c>
       <c r="E23" t="str">
-        <v>IIS TRISNAWATI, S.T., M.T.</v>
+        <v>KARTIKA WATI, ST</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="B24" t="str">
-        <v>7a</v>
+        <v>5</v>
       </c>
       <c r="C24" t="str">
-        <v>2022 - ST 7105 / 07</v>
+        <v>TS 5354</v>
       </c>
       <c r="D24" t="str">
-        <v>Teknologi dan Transformasi Digital</v>
+        <v>Praktikum Surveying dan Sistem Informasi Geografis</v>
       </c>
       <c r="E24" t="str">
-        <v>MUHAMMAD FAIZ SYAIFUL ISLAM, M.Si.</v>
+        <v>KARTIKA WATI, ST</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="B25" t="str">
-        <v>7a</v>
+        <v>5</v>
       </c>
       <c r="C25" t="str">
-        <v>2022 - ST 7106 / 07</v>
+        <v>TS 5355</v>
       </c>
       <c r="D25" t="str">
-        <v>Etika Profesi</v>
+        <v>Rekayasa Sungai dan Pantai</v>
       </c>
       <c r="E25" t="str">
-        <v>Drs. GUNAWAN WIBISONO, M.T.</v>
+        <v>IIS TRISNAWATI, S.T., M.T.</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="B26" t="str">
-        <v>7a</v>
+        <v>5</v>
       </c>
       <c r="C26" t="str">
-        <v>2022 - ST 7107 / 07</v>
+        <v>TS 5356</v>
       </c>
       <c r="D26" t="str">
-        <v>Prasarana dan Sarana PU Terpadu</v>
+        <v>Rekayasa Irigasi dan Rawa</v>
       </c>
       <c r="E26" t="str">
-        <v>PRAYOGA ADHINUGROHO, S.T., M.I.Kom</v>
+        <v>IIS TRISNAWATI, S.T., M.T.</v>
       </c>
     </row>
     <row r="27">
@@ -938,13 +938,13 @@
         <v>7a</v>
       </c>
       <c r="C27" t="str">
-        <v>2022 - ST 7108 / 07</v>
+        <v>ST 7105</v>
       </c>
       <c r="D27" t="str">
-        <v>Rekayasa Sosial</v>
+        <v>Teknologi dan Transformasi Digital</v>
       </c>
       <c r="E27" t="str">
-        <v>Dr. Ir. TIMBUL PM PANJAITAN, MA, M.Th.</v>
+        <v>MUHAMMAD FAIZ SYAIFUL ISLAM, M.Si.</v>
       </c>
     </row>
     <row r="28">
@@ -955,13 +955,13 @@
         <v>7a</v>
       </c>
       <c r="C28" t="str">
-        <v>2022 - ST 7109 / 07</v>
+        <v>ST 7106</v>
       </c>
       <c r="D28" t="str">
-        <v>Sistem Penjamin Mutu Teknik Sipil</v>
+        <v>Etika Profesi</v>
       </c>
       <c r="E28" t="str">
-        <v>DIAN SOVANA, S.T., M.T., IPU.</v>
+        <v>Drs. GUNAWAN WIBISONO, M.T.</v>
       </c>
     </row>
     <row r="29">
@@ -972,13 +972,13 @@
         <v>7a</v>
       </c>
       <c r="C29" t="str">
-        <v>2022 - TS 7363 / 07</v>
+        <v>ST 7107</v>
       </c>
       <c r="D29" t="str">
-        <v>Kewirausahaan Teknik Sipil</v>
+        <v>Prasarana dan Sarana PU Terpadu</v>
       </c>
       <c r="E29" t="str">
-        <v>Ir. BAMBANG TRI SUKMONO, MT</v>
+        <v>PRAYOGA ADHINUGROHO, S.T., M.I.Kom</v>
       </c>
     </row>
     <row r="30">
@@ -989,13 +989,13 @@
         <v>7a</v>
       </c>
       <c r="C30" t="str">
-        <v>2022 - TS 7364 / 07</v>
+        <v>ST 7108</v>
       </c>
       <c r="D30" t="str">
-        <v>Kerja Praktek (KP)</v>
+        <v>Rekayasa Sosial</v>
       </c>
       <c r="E30" t="str">
-        <v/>
+        <v>Dr. Ir. TIMBUL PM PANJAITAN, MA, M.Th.</v>
       </c>
     </row>
     <row r="31">
@@ -1006,13 +1006,13 @@
         <v>7a</v>
       </c>
       <c r="C31" t="str">
-        <v>2022 - TS 7365 / 07</v>
+        <v>ST 7109</v>
       </c>
       <c r="D31" t="str">
-        <v>Perencanaan Jembatan</v>
+        <v>Sistem Penjamin Mutu Teknik Sipil</v>
       </c>
       <c r="E31" t="str">
-        <v>HERI YUGIANTORO, S.T., M.T.</v>
+        <v>DIAN SOVANA, S.T., M.T., IPU.</v>
       </c>
     </row>
     <row r="32">
@@ -1023,13 +1023,13 @@
         <v>7a</v>
       </c>
       <c r="C32" t="str">
-        <v>2022 - TS 7472 / 07</v>
+        <v>TS 7363</v>
       </c>
       <c r="D32" t="str">
-        <v>Perencanaan Bangunan Gedung</v>
+        <v>Kewirausahaan Teknik Sipil</v>
       </c>
       <c r="E32" t="str">
-        <v>Ir. EFFY HIDAYATY, M.T.</v>
+        <v>Ir. BAMBANG TRI SUKMONO, MT</v>
       </c>
     </row>
     <row r="33">
@@ -1037,16 +1037,16 @@
         <v>7</v>
       </c>
       <c r="B33" t="str">
-        <v>7b</v>
+        <v>7a</v>
       </c>
       <c r="C33" t="str">
-        <v>2022 - TS 7473 / 07</v>
+        <v>TS 7364</v>
       </c>
       <c r="D33" t="str">
-        <v>Perencanaan Bangunan SDA</v>
+        <v>Kerja Praktek (KP)</v>
       </c>
       <c r="E33" t="str">
-        <v>HELDY SUHERMAN, S.T., M.S.I</v>
+        <v/>
       </c>
     </row>
     <row r="34">
@@ -1054,16 +1054,16 @@
         <v>7</v>
       </c>
       <c r="B34" t="str">
-        <v>7c</v>
+        <v>7a</v>
       </c>
       <c r="C34" t="str">
-        <v>2022 - TS 7474 / 07</v>
+        <v>TS 7365</v>
       </c>
       <c r="D34" t="str">
-        <v>Perencanaan Bangunan Jalan dan Jembatan</v>
+        <v>Perencanaan Jembatan</v>
       </c>
       <c r="E34" t="str">
-        <v>Dr Ir MUKTAR NAPITUPULU, M.Sc</v>
+        <v>HERI YUGIANTORO, S.T., M.T.</v>
       </c>
     </row>
     <row r="35">
@@ -1074,18 +1074,69 @@
         <v>7a</v>
       </c>
       <c r="C35" t="str">
-        <v>2022 - TS 7476 / 07</v>
+        <v>TS 7472</v>
       </c>
       <c r="D35" t="str">
+        <v>Perencanaan Bangunan Gedung</v>
+      </c>
+      <c r="E35" t="str">
+        <v>Ir. EFFY HIDAYATY, M.T.</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>7</v>
+      </c>
+      <c r="B36" t="str">
+        <v>7b</v>
+      </c>
+      <c r="C36" t="str">
+        <v>TS 7473</v>
+      </c>
+      <c r="D36" t="str">
+        <v>Perencanaan Bangunan SDA</v>
+      </c>
+      <c r="E36" t="str">
+        <v>HELDY SUHERMAN, S.T., M.S.I</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>7</v>
+      </c>
+      <c r="B37" t="str">
+        <v>7c</v>
+      </c>
+      <c r="C37" t="str">
+        <v>TS 7474</v>
+      </c>
+      <c r="D37" t="str">
+        <v>Perencanaan Bangunan Jalan dan Jembatan</v>
+      </c>
+      <c r="E37" t="str">
+        <v>Dr Ir MUKTAR NAPITUPULU, M.Sc</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v>7</v>
+      </c>
+      <c r="B38" t="str">
+        <v>7a</v>
+      </c>
+      <c r="C38" t="str">
+        <v>TS 7476</v>
+      </c>
+      <c r="D38" t="str">
         <v>Manajemen Pemeliharaan Bangunan</v>
       </c>
-      <c r="E35" t="str">
+      <c r="E38" t="str">
         <v>DIAN SOVANA, S.T., M.T., IPU.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E35"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E38"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: link semester 1 & 7 combined courses to slot 7a with integrity check
</commit_message>
<xml_diff>
--- a/data/jadwal_zoom.xlsx
+++ b/data/jadwal_zoom.xlsx
@@ -527,7 +527,7 @@
         <v>1</v>
       </c>
       <c r="B3" t="str">
-        <v>1</v>
+        <v>7a</v>
       </c>
       <c r="C3" t="str">
         <v>PU 1209</v>
@@ -544,7 +544,7 @@
         <v>1</v>
       </c>
       <c r="B4" t="str">
-        <v>1</v>
+        <v>7a</v>
       </c>
       <c r="C4" t="str">
         <v>PU 1210</v>

</xml_diff>